<commit_message>
OTP verification for donor
OTP verification using maitrap.io
</commit_message>
<xml_diff>
--- a/Life/server/data/lifelink_db.xlsx
+++ b/Life/server/data/lifelink_db.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L14"/>
   <sheetData>
     <row r="2">
       <c r="A2" t="str">
@@ -777,13 +777,127 @@
       <c r="K11" t="b">
         <v>1</v>
       </c>
-      <c r="L11" s="1">
+      <c r="L11">
         <v>45984.95185159722</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>69234632a9d7b28957d0eb0c</v>
+      </c>
+      <c r="B12" t="str">
+        <v>mno</v>
+      </c>
+      <c r="C12" t="str">
+        <v>mno@gmail.com</v>
+      </c>
+      <c r="D12" t="str">
+        <v>9481824919</v>
+      </c>
+      <c r="E12" t="str">
+        <v>A+</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Mangalore</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12" t="b">
+        <v>0</v>
+      </c>
+      <c r="J12" t="b">
+        <v>0</v>
+      </c>
+      <c r="K12" t="b">
+        <v>1</v>
+      </c>
+      <c r="L12">
+        <v>45984.96320155093</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>69234680a9d7b28957d0eb11</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Me</v>
+      </c>
+      <c r="C13" t="str">
+        <v>23a43.bhavish@sjec.ac.in</v>
+      </c>
+      <c r="D13" t="str">
+        <v>8904534919</v>
+      </c>
+      <c r="E13" t="str">
+        <v>A+</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Mangalore</v>
+      </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
+      <c r="I13" t="b">
+        <v>0</v>
+      </c>
+      <c r="J13" t="b">
+        <v>0</v>
+      </c>
+      <c r="K13" t="b">
+        <v>1</v>
+      </c>
+      <c r="L13">
+        <v>45984.9641012037</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>6923b7181c52f11af60577df</v>
+      </c>
+      <c r="B14" t="str">
+        <v>mailtrap</v>
+      </c>
+      <c r="C14" t="str">
+        <v>lifelink@system.com</v>
+      </c>
+      <c r="D14" t="str">
+        <v>1234456789</v>
+      </c>
+      <c r="E14" t="str">
+        <v>A+</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Mangalore</v>
+      </c>
+      <c r="G14">
+        <v>0</v>
+      </c>
+      <c r="H14">
+        <v>0</v>
+      </c>
+      <c r="I14" t="b">
+        <v>0</v>
+      </c>
+      <c r="J14" t="b">
+        <v>0</v>
+      </c>
+      <c r="K14" t="b">
+        <v>1</v>
+      </c>
+      <c r="L14" s="1">
+        <v>45985.297717719906</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L14"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>